<commit_message>
Add reminder mode support to task import
</commit_message>
<xml_diff>
--- a/src/public/templates/tasks_import_template.xlsx
+++ b/src/public/templates/tasks_import_template.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gustavo.benicio\Documents\Projeto FTA\src\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larissa.bittar/Documents/GitHub/fta/src/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E347BA42-021D-408F-B578-067888F849FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E2AFB7-6232-C04B-90E7-D791E21941DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38880" yWindow="5360" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
     <sheet name="Planilha1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tasks!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Título*</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>ID Slack de quem delegou</t>
+  </si>
+  <si>
+    <t>Tipo de Prazo*</t>
   </si>
 </sst>
 </file>
@@ -141,6 +144,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -521,22 +525,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27" customWidth="1"/>
-    <col min="6" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="21" customWidth="1"/>
-    <col min="13" max="13" width="23" customWidth="1"/>
+    <col min="6" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="19" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="13" width="21" customWidth="1"/>
+    <col min="14" max="14" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -562,52 +566,65 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I5" xr:uid="{643024B8-E6DA-44DD-9CBB-AB6A380CADF4}">
+  <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J5" xr:uid="{643024B8-E6DA-44DD-9CBB-AB6A380CADF4}">
       <formula1>"none,daily,weekly,monthly,quarterly,semiannual,annual"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H2:H5" xr:uid="{1F82843B-206A-40B9-8595-0BD162EC5DA6}">
       <formula1>"light,asap,turbo"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I1048576" xr:uid="{D62227E9-6051-EC43-A614-77094012C375}">
+      <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x12ac">
+          <x12ac:list>"até, a partir"</x12ac:list>
+        </mc:Choice>
+        <mc:Fallback>
+          <formula1>"até, a partir"</formula1>
+        </mc:Fallback>
+      </mc:AlternateContent>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -617,62 +634,62 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329E06CA-2CA0-4676-B541-8DD8C6504178}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="74.109375" customWidth="1"/>
+    <col min="1" max="1" width="74.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="20" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" ht="20" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>21</v>
       </c>

</xml_diff>